<commit_message>
Remove Data sources / Data quality pages, Makeen/Incorta and the Unassigned Amanah; real SADAD biller ids; exclusions reference
- Delete the Data sources and Data quality settings pages (routes redirect to the Metric dictionary); re-point their links.
- Remove Makeen and Incorta and the "Unassigned" Amanah everywhere (catalog, engine, world, reports, Decision Room, planning, map); the deterministic world keeps its random draws and an inert internal set so stable enforcement-order ids do not move. Delete dead sourceMap.js and ledgerImport.js.
- Invoice ids use the real SADAD biller ids (Ministry 177; Riyadh 010 ...); Hafr Al-Batin keeps a marked demo placeholder. Samples regenerated.
- Metric dictionary > Metrics: add the SADAD-number/biller-id example and the exclusions list reference (21 Oct 2026 session).
- Tests updated (162 pass); dist and api bundle rebuilt.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/dist/samples/exclusion-upload-sample.xlsx
+++ b/dist/samples/exclusion-upload-sample.xlsx
@@ -480,19 +480,19 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>177-409260122511</v>
+        <v>177-407500123303</v>
       </c>
       <c r="B4" t="str">
-        <v>2026-03-13</v>
+        <v>2026-01-08</v>
       </c>
       <c r="C4">
-        <v>20695750</v>
+        <v>83462690</v>
       </c>
       <c r="D4" t="str">
-        <v>أمانة محافظة جدة</v>
+        <v>أمانة منطقة عسير</v>
       </c>
       <c r="E4" t="str">
-        <v>شركة بنيان للمقاولات</v>
+        <v>مجموعة الخليج للخدمات</v>
       </c>
       <c r="F4" t="str">
         <v>1438001</v>
@@ -526,22 +526,22 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>177-411320121584</v>
+        <v>177-411220121629</v>
       </c>
       <c r="B6" t="str">
-        <v>2026-05-28</v>
+        <v>2026-05-29</v>
       </c>
       <c r="C6">
-        <v>6579780</v>
+        <v>21569420</v>
       </c>
       <c r="D6" t="str">
-        <v>أمانة المنطقة الشرقية</v>
+        <v>أمانة محافظة جدة</v>
       </c>
       <c r="E6" t="str">
-        <v>شركة الخليج للنقل</v>
+        <v>شركة الأفق للتطوير</v>
       </c>
       <c r="F6" t="str">
-        <v>142163</v>
+        <v>142113</v>
       </c>
       <c r="G6" t="str">
         <v>التعديات واستغلال المواقع (محضر التعدي)</v>
@@ -549,22 +549,22 @@
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>177-412200121188</v>
+        <v>177-411540121485</v>
       </c>
       <c r="B7" t="str">
-        <v>2026-07-20</v>
+        <v>2026-06-04</v>
       </c>
       <c r="C7">
-        <v>17307570</v>
+        <v>222557380</v>
       </c>
       <c r="D7" t="str">
-        <v>أمانة محافظة جدة</v>
+        <v>أمانة منطقة عسير</v>
       </c>
       <c r="E7" t="str">
-        <v>شركة القمة للتطوير</v>
+        <v>مجموعة آفاق للنقل</v>
       </c>
       <c r="F7" t="str">
-        <v>1438001</v>
+        <v>1438002</v>
       </c>
       <c r="G7" t="str">
         <v>إفادات الأمانات</v>
@@ -575,19 +575,19 @@
         <v>177-880000071271</v>
       </c>
       <c r="B8" t="str">
-        <v>2025-03-09</v>
+        <v>2025-03-07</v>
       </c>
       <c r="C8">
-        <v>211460090</v>
+        <v>2858610</v>
       </c>
       <c r="D8" t="str">
         <v>أمانة محافظة جدة</v>
       </c>
       <c r="E8" t="str">
-        <v>مجموعة المنارة للتموين</v>
+        <v>مجموعة الشروق للاستثمار</v>
       </c>
       <c r="F8" t="str">
-        <v>14155</v>
+        <v>1438001</v>
       </c>
       <c r="G8" t="str">
         <v>إفادات الأمانات</v>
@@ -595,22 +595,22 @@
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>177-410810121854</v>
+        <v>177-410770121872</v>
       </c>
       <c r="B9" t="str">
-        <v>2025-06-03</v>
+        <v>2025-06-13</v>
       </c>
       <c r="C9">
-        <v>45909540</v>
+        <v>10220080</v>
       </c>
       <c r="D9" t="str">
         <v>أمانة محافظة جدة</v>
       </c>
       <c r="E9" t="str">
-        <v>شركة الفجر للإعلان</v>
+        <v>شركة بوابة للمقاولات</v>
       </c>
       <c r="F9" t="str">
-        <v>1438002</v>
+        <v>1438</v>
       </c>
       <c r="G9" t="str">
         <v>إفادات الأمانات</v>
@@ -618,22 +618,22 @@
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>177-413700120513</v>
+        <v>177-413620120549</v>
       </c>
       <c r="B10" t="str">
-        <v>2026-09-28</v>
+        <v>2026-09-21</v>
       </c>
       <c r="C10">
-        <v>4981940</v>
+        <v>13818250</v>
       </c>
       <c r="D10" t="str">
         <v>أمانة محافظة جدة</v>
       </c>
       <c r="E10" t="str">
-        <v>مجموعة الواحة للمقاولات</v>
+        <v>مؤسسة النخبة للاستثمار</v>
       </c>
       <c r="F10" t="str">
-        <v>1438</v>
+        <v>1438001</v>
       </c>
       <c r="G10" t="str">
         <v>التعديات واستغلال المواقع (محضر التعدي)</v>
@@ -687,22 +687,22 @@
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>177-409320122484</v>
+        <v>177-408940122655</v>
       </c>
       <c r="B13" t="str">
-        <v>2026-03-24</v>
+        <v>2026-02-15</v>
       </c>
       <c r="C13">
-        <v>36602400</v>
+        <v>15448310</v>
       </c>
       <c r="D13" t="str">
-        <v>أمانة محافظة جدة</v>
+        <v>أمانة منطقة مكة المكرمة</v>
       </c>
       <c r="E13" t="str">
-        <v>مؤسسة السحاب التجارية</v>
+        <v>مجموعة الخليج للنقل</v>
       </c>
       <c r="F13" t="str">
-        <v>1438001</v>
+        <v>11442</v>
       </c>
       <c r="G13" t="str">
         <v>إفادات الأمانات</v>
@@ -756,22 +756,22 @@
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>177-412720120954</v>
+        <v>177-412000121278</v>
       </c>
       <c r="B16" t="str">
-        <v>2026-07-20</v>
+        <v>2026-06-20</v>
       </c>
       <c r="C16">
-        <v>22216500</v>
+        <v>8835840</v>
       </c>
       <c r="D16" t="str">
         <v>أمانة محافظة جدة</v>
       </c>
       <c r="E16" t="str">
-        <v>شركة الأفق للتطوير</v>
+        <v>مؤسسة الأفق التجارية</v>
       </c>
       <c r="F16" t="str">
-        <v>142113</v>
+        <v>142163</v>
       </c>
       <c r="G16" t="str">
         <v>إفادات الأمانات</v>
@@ -782,19 +782,19 @@
         <v>177-880000087109</v>
       </c>
       <c r="B17" t="str">
-        <v>2025-03-09</v>
+        <v>2025-03-28</v>
       </c>
       <c r="C17">
-        <v>66992670</v>
+        <v>42545000</v>
       </c>
       <c r="D17" t="str">
-        <v>أمانة منطقة عسير</v>
+        <v>أمانة منطقة الحدود الشمالية</v>
       </c>
       <c r="E17" t="str">
-        <v>مجموعة النخبة للمقاولات</v>
+        <v>شركة بوابة للخدمات</v>
       </c>
       <c r="F17" t="str">
-        <v>142163</v>
+        <v>14155</v>
       </c>
       <c r="G17" t="str">
         <v>إفادات الأمانات</v>
@@ -802,22 +802,22 @@
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>177-411490121548</v>
+        <v>177-411410121584</v>
       </c>
       <c r="B18" t="str">
-        <v>2025-07-12</v>
+        <v>2025-07-01</v>
       </c>
       <c r="C18">
-        <v>18038390</v>
+        <v>47036730</v>
       </c>
       <c r="D18" t="str">
-        <v>أمانة محافظة جدة</v>
+        <v>أمانة منطقة الرياض</v>
       </c>
       <c r="E18" t="str">
-        <v>شركة بوابة للمقاولات</v>
+        <v>مجموعة الخليج العقارية</v>
       </c>
       <c r="F18" t="str">
-        <v>1438002</v>
+        <v>1438001</v>
       </c>
       <c r="G18" t="str">
         <v>إفادات الأمانات</v>
@@ -848,22 +848,22 @@
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>177-410670121917</v>
+        <v>177-410030122205</v>
       </c>
       <c r="B20" t="str">
-        <v>2025-05-09</v>
+        <v>2025-04-09</v>
       </c>
       <c r="C20">
-        <v>66992670</v>
+        <v>217803890</v>
       </c>
       <c r="D20" t="str">
-        <v>أمانة منطقة عسير</v>
+        <v>أمانة محافظة جدة</v>
       </c>
       <c r="E20" t="str">
-        <v>مؤسسة الصقر للتطوير</v>
+        <v>شركة الأفق للتطوير</v>
       </c>
       <c r="F20" t="str">
-        <v>142163</v>
+        <v>14155</v>
       </c>
       <c r="G20" t="str">
         <v>التعديات واستغلال المواقع (محضر التعدي)</v>
@@ -871,22 +871,22 @@
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>177-410670121917</v>
+        <v>177-410030122205</v>
       </c>
       <c r="B21" t="str">
-        <v>2025-05-09</v>
+        <v>2025-04-09</v>
       </c>
       <c r="C21">
-        <v>66992670</v>
+        <v>217803890</v>
       </c>
       <c r="D21" t="str">
-        <v>أمانة منطقة عسير</v>
+        <v>أمانة محافظة جدة</v>
       </c>
       <c r="E21" t="str">
-        <v>مؤسسة الصقر للتطوير</v>
+        <v>شركة الأفق للتطوير</v>
       </c>
       <c r="F21" t="str">
-        <v>142163</v>
+        <v>14155</v>
       </c>
       <c r="G21" t="str">
         <v>سبب غير معروف</v>
@@ -894,22 +894,22 @@
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>177-409920122214</v>
+        <v>177-409280122502</v>
       </c>
       <c r="B22" t="str">
-        <v>2026-04-21</v>
+        <v>2026-03-12</v>
       </c>
       <c r="C22">
-        <v>35451360</v>
+        <v>149461930</v>
       </c>
       <c r="D22" t="str">
         <v>أمانة محافظة جدة</v>
       </c>
       <c r="E22" t="str">
-        <v>شركة الرؤية للإعلان</v>
+        <v>مؤسسة المنارة للخدمات</v>
       </c>
       <c r="F22" t="str">
-        <v>1438</v>
+        <v>1438002</v>
       </c>
       <c r="G22" t="str">
         <v>إفادات الأمانات</v>
@@ -917,7 +917,7 @@
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>301-407600123339</v>
+        <v>010-407600123339</v>
       </c>
       <c r="B23" t="str">
         <v>2024-10-14</v>
@@ -963,22 +963,22 @@
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>177-412780120927</v>
+        <v>177-412160121206</v>
       </c>
       <c r="B25" t="str">
-        <v>2026-07-18</v>
+        <v>2026-07-20</v>
       </c>
       <c r="C25">
-        <v>46623390</v>
+        <v>77693490</v>
       </c>
       <c r="D25" t="str">
-        <v>أمانة المدينة المنورة</v>
+        <v>أمانة محافظة جدة</v>
       </c>
       <c r="E25" t="str">
-        <v>شركة القمة التجارية</v>
+        <v>شركة الندى للاستثمار</v>
       </c>
       <c r="F25" t="str">
-        <v>14155</v>
+        <v>1438001</v>
       </c>
       <c r="G25" t="str">
         <v>إفادات الأمانات</v>
@@ -989,19 +989,19 @@
         <v>177-880000102947</v>
       </c>
       <c r="B26" t="str">
-        <v>2025-04-02</v>
+        <v>2025-03-28</v>
       </c>
       <c r="C26">
-        <v>8364210</v>
+        <v>6388130</v>
       </c>
       <c r="D26" t="str">
         <v>أمانة المنطقة الشرقية</v>
       </c>
       <c r="E26" t="str">
-        <v>مؤسسة المدار للنقل</v>
+        <v>شركة الخليج للنقل</v>
       </c>
       <c r="F26" t="str">
-        <v>1438</v>
+        <v>142163</v>
       </c>
       <c r="G26" t="str">
         <v>إفادات الأمانات</v>
@@ -1009,22 +1009,22 @@
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>177-412850120936</v>
+        <v>177-411690121458</v>
       </c>
       <c r="B27" t="str">
-        <v>2025-09-24</v>
+        <v>2025-07-30</v>
       </c>
       <c r="C27">
-        <v>17286710</v>
+        <v>80617220</v>
       </c>
       <c r="D27" t="str">
-        <v>أمانة منطقة عسير</v>
+        <v>أمانة منطقة الرياض</v>
       </c>
       <c r="E27" t="str">
-        <v>مجموعة الدرة للإعلان</v>
+        <v>مؤسسة الفجر التجارية</v>
       </c>
       <c r="F27" t="str">
-        <v>1438002</v>
+        <v>11442</v>
       </c>
       <c r="G27" t="str">
         <v>إفادات الأمانات</v>
@@ -1055,19 +1055,19 @@
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>177-412030121305</v>
+        <v>177-410690121908</v>
       </c>
       <c r="B29" t="str">
-        <v>2025-07-28</v>
+        <v>2025-05-28</v>
       </c>
       <c r="C29">
         <v>6388130</v>
       </c>
       <c r="D29" t="str">
-        <v>أمانة المنطقة الشرقية</v>
+        <v>أمانة محافظة جدة</v>
       </c>
       <c r="E29" t="str">
-        <v>شركة الخليج للنقل</v>
+        <v>شركة الأفق للتطوير</v>
       </c>
       <c r="F29" t="str">
         <v>142163</v>
@@ -1078,10 +1078,10 @@
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>177-412030121305</v>
+        <v>177-410690121908</v>
       </c>
       <c r="B30" t="str">
-        <v>2025-07-28</v>
+        <v>2025-05-28</v>
       </c>
       <c r="C30">
         <v>6388130</v>
@@ -1090,7 +1090,7 @@
         <v>أمانة غير معروفة</v>
       </c>
       <c r="E30" t="str">
-        <v>شركة الخليج للنقل</v>
+        <v>شركة الأفق للتطوير</v>
       </c>
       <c r="F30" t="str">
         <v>142163</v>
@@ -1101,19 +1101,19 @@
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>177-410000122178</v>
+        <v>177-409340122475</v>
       </c>
       <c r="B31" t="str">
-        <v>2026-04-06</v>
+        <v>2026-03-18</v>
       </c>
       <c r="C31">
-        <v>57345075</v>
+        <v>77837315</v>
       </c>
       <c r="D31" t="str">
-        <v>أمانة محافظة جدة</v>
+        <v>أمانة المنطقة الشرقية</v>
       </c>
       <c r="E31" t="str">
-        <v>مؤسسة المدار للتطوير</v>
+        <v>شركة واحة التجارية</v>
       </c>
       <c r="F31" t="str">
         <v>1438</v>
@@ -1124,7 +1124,7 @@
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>303-407640123321</v>
+        <v>025-407640123321</v>
       </c>
       <c r="B32" t="str">
         <v>2024-10-13</v>
@@ -1170,19 +1170,19 @@
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>177-412840120900</v>
+        <v>177-412200121188</v>
       </c>
       <c r="B34" t="str">
-        <v>2026-08-18</v>
+        <v>2026-07-29</v>
       </c>
       <c r="C34">
-        <v>11726880</v>
+        <v>17307570</v>
       </c>
       <c r="D34" t="str">
-        <v>أمانة منطقة الرياض</v>
+        <v>أمانة محافظة جدة</v>
       </c>
       <c r="E34" t="str">
-        <v>مجموعة آفاق للخدمات</v>
+        <v>شركة القمة للتطوير</v>
       </c>
       <c r="F34" t="str">
         <v>9999999</v>
@@ -1196,19 +1196,19 @@
         <v>177-880000118785</v>
       </c>
       <c r="B35" t="str">
-        <v>2025-05-05</v>
+        <v>2025-04-29</v>
       </c>
       <c r="C35">
-        <v>66118220</v>
+        <v>3787410</v>
       </c>
       <c r="D35" t="str">
         <v>أمانة محافظة جدة</v>
       </c>
       <c r="E35" t="str">
-        <v>شركة الرمال العقارية</v>
+        <v>مجموعة نماء للتطوير</v>
       </c>
       <c r="F35" t="str">
-        <v>1438002</v>
+        <v>11452105</v>
       </c>
       <c r="G35" t="str">
         <v>إفادات الأمانات</v>
@@ -1216,22 +1216,22 @@
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>177-413190120783</v>
+        <v>177-412850120936</v>
       </c>
       <c r="B36" t="str">
-        <v>2025-09-22</v>
+        <v>2025-09-24</v>
       </c>
       <c r="C36">
-        <v>599230</v>
+        <v>17286710</v>
       </c>
       <c r="D36" t="str">
-        <v>أمانة المنطقة الشرقية</v>
+        <v>أمانة منطقة عسير</v>
       </c>
       <c r="E36" t="str">
-        <v>شركة الندى للخدمات</v>
+        <v>مجموعة الدرة للإعلان</v>
       </c>
       <c r="F36" t="str">
-        <v>11422</v>
+        <v>1438002</v>
       </c>
       <c r="G36" t="str">
         <v>إفادات الأمانات</v>
@@ -1262,19 +1262,19 @@
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>177-413970120432</v>
+        <v>177-412030121305</v>
       </c>
       <c r="B38" t="str">
-        <v>2025-10-09</v>
+        <v>2025-07-28</v>
       </c>
       <c r="C38">
-        <v>66992670</v>
+        <v>6388130</v>
       </c>
       <c r="D38" t="str">
-        <v>أمانة منطقة عسير</v>
+        <v>أمانة المنطقة الشرقية</v>
       </c>
       <c r="E38" t="str">
-        <v>مجموعة النخبة للمقاولات</v>
+        <v>شركة الخليج للنقل</v>
       </c>
       <c r="F38" t="str">
         <v>142163</v>
@@ -1308,22 +1308,22 @@
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>177-410440121980</v>
+        <v>177-409960122196</v>
       </c>
       <c r="B40" t="str">
-        <v>2026-04-25</v>
+        <v>2026-04-22</v>
       </c>
       <c r="C40">
-        <v>18317335</v>
+        <v>6077835</v>
       </c>
       <c r="D40" t="str">
         <v>أمانة محافظة جدة</v>
       </c>
       <c r="E40" t="str">
-        <v>مؤسسة الدرة للنقل</v>
+        <v>شركة الرؤية للاستثمار</v>
       </c>
       <c r="F40" t="str">
-        <v>11422</v>
+        <v>1438001</v>
       </c>
       <c r="G40" t="str">
         <v>إفادات الأمانات</v>
@@ -1354,19 +1354,19 @@
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>177-408570122862</v>
+        <v>177-408510122889</v>
       </c>
       <c r="B42" t="str">
-        <v>2025-02-28</v>
+        <v>2025-02-01</v>
       </c>
       <c r="C42">
-        <v>4164930</v>
+        <v>9600950</v>
       </c>
       <c r="D42" t="str">
-        <v>أمانة منطقة جازان</v>
+        <v>أمانة محافظة جدة</v>
       </c>
       <c r="E42" t="str">
-        <v>شركة الواحة للاستثمار</v>
+        <v>مجموعة الرؤية التجارية</v>
       </c>
       <c r="F42" t="str">
         <v>11442</v>
@@ -1377,19 +1377,19 @@
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>177-413040120810</v>
+        <v>177-412720120954</v>
       </c>
       <c r="B43" t="str">
-        <v>2026-08-18</v>
+        <v>2026-07-29</v>
       </c>
       <c r="C43">
-        <v>14303970</v>
+        <v>22216500</v>
       </c>
       <c r="D43" t="str">
-        <v>أمانة محافظة الطائف</v>
+        <v>أمانة محافظة جدة</v>
       </c>
       <c r="E43" t="str">
-        <v>مجموعة الرمال للتموين</v>
+        <v>شركة الأفق للتطوير</v>
       </c>
       <c r="F43" t="str">
         <v>9999999</v>
@@ -1403,16 +1403,16 @@
         <v>177-880000134623</v>
       </c>
       <c r="B44" t="str">
-        <v>2025-05-09</v>
+        <v>2025-05-05</v>
       </c>
       <c r="C44">
-        <v>43823000</v>
+        <v>66118220</v>
       </c>
       <c r="D44" t="str">
-        <v>أمانة منطقة عسير</v>
+        <v>أمانة محافظة جدة</v>
       </c>
       <c r="E44" t="str">
-        <v>مؤسسة الصقر للتطوير</v>
+        <v>شركة الرمال العقارية</v>
       </c>
       <c r="F44" t="str">
         <v>1438002</v>
@@ -1423,22 +1423,22 @@
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>177-414050120396</v>
+        <v>177-413190120783</v>
       </c>
       <c r="B45" t="str">
-        <v>2025-11-27</v>
+        <v>2025-09-22</v>
       </c>
       <c r="C45">
-        <v>7107220</v>
+        <v>599230</v>
       </c>
       <c r="D45" t="str">
-        <v>أمانة محافظة جدة</v>
+        <v>أمانة المنطقة الشرقية</v>
       </c>
       <c r="E45" t="str">
-        <v>شركة بوابة للخدمات</v>
+        <v>شركة الندى للخدمات</v>
       </c>
       <c r="F45" t="str">
-        <v>1438002</v>
+        <v>11422</v>
       </c>
       <c r="G45" t="str">
         <v>إفادات الأمانات</v>
@@ -1446,19 +1446,19 @@
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>177-408570122862</v>
+        <v>177-408510122889</v>
       </c>
       <c r="B46" t="str">
-        <v>2025-02-28</v>
+        <v>2025-02-01</v>
       </c>
       <c r="C46">
-        <v>4164930</v>
+        <v>9600950</v>
       </c>
       <c r="D46" t="str">
-        <v>أمانة منطقة الحدود الشمالية</v>
+        <v>أمانة المدينة المنورة</v>
       </c>
       <c r="E46" t="str">
-        <v>شركة الواحة للاستثمار</v>
+        <v>مجموعة الرؤية التجارية</v>
       </c>
       <c r="F46" t="str">
         <v>11442</v>
@@ -1469,10 +1469,10 @@
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v>177-415370119802</v>
+        <v>177-413970120432</v>
       </c>
       <c r="B47" t="str">
-        <v>2025-12-09</v>
+        <v>2025-10-09</v>
       </c>
       <c r="C47">
         <v>66992670</v>
@@ -1492,22 +1492,22 @@
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>177-410960121746</v>
+        <v>177-410180122097</v>
       </c>
       <c r="B48" t="str">
-        <v>2026-05-30</v>
+        <v>2026-04-22</v>
       </c>
       <c r="C48">
-        <v>7546875</v>
+        <v>25785775</v>
       </c>
       <c r="D48" t="str">
-        <v>أمانة المنطقة الشرقية</v>
+        <v>أمانة محافظة جدة</v>
       </c>
       <c r="E48" t="str">
-        <v>مؤسسة الريادة للإعلان</v>
+        <v>مجموعة الواحة للإعلان</v>
       </c>
       <c r="F48" t="str">
-        <v>11100-11105</v>
+        <v>11114</v>
       </c>
       <c r="G48" t="str">
         <v>إفادات الأمانات</v>
@@ -1538,22 +1538,22 @@
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v>177-409630122385</v>
+        <v>177-408930122700</v>
       </c>
       <c r="B50" t="str">
-        <v>2025-04-02</v>
+        <v>2025-03-07</v>
       </c>
       <c r="C50">
-        <v>8364210</v>
+        <v>2858610</v>
       </c>
       <c r="D50" t="str">
-        <v>أمانة المنطقة الشرقية</v>
+        <v>أمانة محافظة جدة</v>
       </c>
       <c r="E50" t="str">
-        <v>مؤسسة المدار للنقل</v>
+        <v>مجموعة الشروق للاستثمار</v>
       </c>
       <c r="F50" t="str">
-        <v>1438</v>
+        <v>1438001</v>
       </c>
       <c r="G50" t="str">
         <v>إفادات الأمانات</v>
@@ -1561,19 +1561,19 @@
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>177-413460120621</v>
+        <v>177-412780120927</v>
       </c>
       <c r="B51" t="str">
-        <v>2026-08-30</v>
+        <v>2026-07-27</v>
       </c>
       <c r="C51">
-        <v>8835840</v>
+        <v>46623390</v>
       </c>
       <c r="D51" t="str">
-        <v>أمانة محافظة جدة</v>
+        <v>أمانة المدينة المنورة</v>
       </c>
       <c r="E51" t="str">
-        <v>مؤسسة الأفق التجارية</v>
+        <v>شركة القمة التجارية</v>
       </c>
       <c r="F51" t="str">
         <v>9999999</v>
@@ -1590,7 +1590,7 @@
         <v>2025-05-09</v>
       </c>
       <c r="C52">
-        <v>66992670</v>
+        <v>43823000</v>
       </c>
       <c r="D52" t="str">
         <v>أمانة منطقة عسير</v>
@@ -1599,7 +1599,7 @@
         <v>مؤسسة الصقر للتطوير</v>
       </c>
       <c r="F52" t="str">
-        <v>142163</v>
+        <v>1438002</v>
       </c>
       <c r="G52" t="str">
         <v>إفادات الأمانات</v>
@@ -1607,22 +1607,22 @@
     </row>
     <row r="53">
       <c r="A53" t="str">
-        <v>177-414270120297</v>
+        <v>177-414050120396</v>
       </c>
       <c r="B53" t="str">
-        <v>2025-11-28</v>
+        <v>2025-11-27</v>
       </c>
       <c r="C53">
-        <v>11989680</v>
+        <v>7107220</v>
       </c>
       <c r="D53" t="str">
-        <v>أمانة المنطقة الشرقية</v>
+        <v>أمانة محافظة جدة</v>
       </c>
       <c r="E53" t="str">
-        <v>شركة الفجر للتموين</v>
+        <v>شركة بوابة للخدمات</v>
       </c>
       <c r="F53" t="str">
-        <v>11114</v>
+        <v>1438002</v>
       </c>
       <c r="G53" t="str">
         <v>إفادات الأمانات</v>
@@ -1630,22 +1630,22 @@
     </row>
     <row r="54">
       <c r="A54" t="str">
-        <v>177-409630122385</v>
+        <v>177-408930122700</v>
       </c>
       <c r="B54" t="str">
-        <v>2025-04-02</v>
+        <v>2025-03-07</v>
       </c>
       <c r="C54">
-        <v>8364210</v>
+        <v>2858610</v>
       </c>
       <c r="D54" t="str">
-        <v>أمانة منطقة عسير</v>
+        <v>أمانة المدينة المنورة</v>
       </c>
       <c r="E54" t="str">
-        <v>مؤسسة المدار للنقل</v>
+        <v>مجموعة الشروق للاستثمار</v>
       </c>
       <c r="F54" t="str">
-        <v>1438</v>
+        <v>1438001</v>
       </c>
       <c r="G54" t="str">
         <v>إفادات الأمانات</v>
@@ -1653,22 +1653,22 @@
     </row>
     <row r="55">
       <c r="A55" t="str">
-        <v>177-409060122601</v>
+        <v>177-415370119802</v>
       </c>
       <c r="B55" t="str">
-        <v>2026-02-26</v>
+        <v>2025-12-09</v>
       </c>
       <c r="C55">
-        <v>21569420</v>
+        <v>66992670</v>
       </c>
       <c r="D55" t="str">
-        <v>أمانة محافظة جدة</v>
+        <v>أمانة منطقة عسير</v>
       </c>
       <c r="E55" t="str">
-        <v>شركة الأفق للتطوير</v>
+        <v>مجموعة النخبة للمقاولات</v>
       </c>
       <c r="F55" t="str">
-        <v>142113</v>
+        <v>142163</v>
       </c>
       <c r="G55" t="str">
         <v>التعديات واستغلال المواقع (محضر التعدي)</v>
@@ -1676,22 +1676,22 @@
     </row>
     <row r="56">
       <c r="A56" t="str">
-        <v>177-411560121476</v>
+        <v>177-410940121755</v>
       </c>
       <c r="B56" t="str">
-        <v>2026-06-02</v>
+        <v>2026-05-26</v>
       </c>
       <c r="C56">
-        <v>1108165</v>
+        <v>75106725</v>
       </c>
       <c r="D56" t="str">
-        <v>أمانة محافظة الطائف</v>
+        <v>أمانة محافظة جدة</v>
       </c>
       <c r="E56" t="str">
-        <v>مجموعة المدار للتموين</v>
+        <v>مؤسسة الندى العقارية</v>
       </c>
       <c r="F56" t="str">
-        <v>1438</v>
+        <v>1421909</v>
       </c>
       <c r="G56" t="str">
         <v>إفادات الأمانات</v>
@@ -1722,22 +1722,22 @@
     </row>
     <row r="58">
       <c r="A58" t="str">
-        <v>177-410130122160</v>
+        <v>177-409730122340</v>
       </c>
       <c r="B58" t="str">
-        <v>2025-05-05</v>
+        <v>2025-04-29</v>
       </c>
       <c r="C58">
-        <v>66118220</v>
+        <v>3787410</v>
       </c>
       <c r="D58" t="str">
         <v>أمانة محافظة جدة</v>
       </c>
       <c r="E58" t="str">
-        <v>شركة الرمال العقارية</v>
+        <v>مجموعة نماء للتطوير</v>
       </c>
       <c r="F58" t="str">
-        <v>1438002</v>
+        <v>11452105</v>
       </c>
       <c r="G58" t="str">
         <v>إفادات الأمانات</v>
@@ -1745,19 +1745,19 @@
     </row>
     <row r="59">
       <c r="A59" t="str">
-        <v>177-413540120585</v>
+        <v>177-412840120900</v>
       </c>
       <c r="B59" t="str">
-        <v>2026-08-28</v>
+        <v>2026-08-18</v>
       </c>
       <c r="C59">
-        <v>6579780</v>
+        <v>11726880</v>
       </c>
       <c r="D59" t="str">
-        <v>أمانة المنطقة الشرقية</v>
+        <v>أمانة منطقة الرياض</v>
       </c>
       <c r="E59" t="str">
-        <v>شركة الخليج للنقل</v>
+        <v>مجموعة آفاق للخدمات</v>
       </c>
       <c r="F59" t="str">
         <v>9999999</v>
@@ -1771,19 +1771,19 @@
         <v>177-880000166299</v>
       </c>
       <c r="B60" t="str">
-        <v>2025-06-03</v>
+        <v>2025-05-09</v>
       </c>
       <c r="C60">
-        <v>45909540</v>
+        <v>66992670</v>
       </c>
       <c r="D60" t="str">
-        <v>أمانة محافظة جدة</v>
+        <v>أمانة منطقة عسير</v>
       </c>
       <c r="E60" t="str">
-        <v>شركة الفجر للإعلان</v>
+        <v>مؤسسة الصقر للتطوير</v>
       </c>
       <c r="F60" t="str">
-        <v>1438002</v>
+        <v>142163</v>
       </c>
       <c r="G60" t="str">
         <v>إفادات الأمانات</v>
@@ -1791,22 +1791,22 @@
     </row>
     <row r="61">
       <c r="A61" t="str">
-        <v>177-415090119928</v>
+        <v>177-414270120297</v>
       </c>
       <c r="B61" t="str">
-        <v>2025-12-17</v>
+        <v>2025-11-28</v>
       </c>
       <c r="C61">
-        <v>26746230</v>
+        <v>11989680</v>
       </c>
       <c r="D61" t="str">
-        <v>أمانة المدينة المنورة</v>
+        <v>أمانة المنطقة الشرقية</v>
       </c>
       <c r="E61" t="str">
-        <v>شركة الصقر للإعلان</v>
+        <v>شركة الفجر للتموين</v>
       </c>
       <c r="F61" t="str">
-        <v>11442</v>
+        <v>11114</v>
       </c>
       <c r="G61" t="str">
         <v>إفادات الأمانات</v>
@@ -1837,22 +1837,22 @@
     </row>
     <row r="63">
       <c r="A63" t="str">
-        <v>177-410660121881</v>
+        <v>177-409060122601</v>
       </c>
       <c r="B63" t="str">
-        <v>2026-04-27</v>
+        <v>2026-02-26</v>
       </c>
       <c r="C63">
-        <v>6579780</v>
+        <v>21569420</v>
       </c>
       <c r="D63" t="str">
-        <v>أمانة المنطقة الشرقية</v>
+        <v>أمانة محافظة جدة</v>
       </c>
       <c r="E63" t="str">
-        <v>شركة الخليج للنقل</v>
+        <v>شركة الأفق للتطوير</v>
       </c>
       <c r="F63" t="str">
-        <v>142163</v>
+        <v>142113</v>
       </c>
       <c r="G63" t="str">
         <v>التعديات واستغلال المواقع (محضر التعدي)</v>
@@ -1860,22 +1860,22 @@
     </row>
     <row r="64">
       <c r="A64" t="str">
-        <v>177-412080121242</v>
+        <v>177-411260121611</v>
       </c>
       <c r="B64" t="str">
-        <v>2026-06-18</v>
+        <v>2026-05-19</v>
       </c>
       <c r="C64">
-        <v>6579780</v>
+        <v>43821350</v>
       </c>
       <c r="D64" t="str">
-        <v>أمانة المنطقة الشرقية</v>
+        <v>أمانة منطقة الحدود الشمالية</v>
       </c>
       <c r="E64" t="str">
-        <v>شركة الخليج للنقل</v>
+        <v>شركة بوابة للخدمات</v>
       </c>
       <c r="F64" t="str">
-        <v>142163</v>
+        <v>14155</v>
       </c>
       <c r="G64" t="str">
         <v>إفادات الأمانات</v>
@@ -1886,19 +1886,19 @@
         <v>177-880000047514</v>
       </c>
       <c r="B65" t="str">
-        <v>2025-02-01</v>
+        <v>2025-02-23</v>
       </c>
       <c r="C65">
-        <v>9600950</v>
+        <v>33373590</v>
       </c>
       <c r="D65" t="str">
         <v>أمانة محافظة جدة</v>
       </c>
       <c r="E65" t="str">
-        <v>مجموعة الرؤية التجارية</v>
+        <v>مجموعة النخبة للتشغيل</v>
       </c>
       <c r="F65" t="str">
-        <v>11442</v>
+        <v>1421909</v>
       </c>
       <c r="G65" t="str">
         <v>إفادات الأمانات</v>
@@ -1906,22 +1906,22 @@
     </row>
     <row r="66">
       <c r="A66" t="str">
-        <v>177-410230122115</v>
+        <v>177-410170122142</v>
       </c>
       <c r="B66" t="str">
-        <v>2025-05-09</v>
+        <v>2025-05-29</v>
       </c>
       <c r="C66">
-        <v>43823000</v>
+        <v>17067910</v>
       </c>
       <c r="D66" t="str">
-        <v>أمانة منطقة عسير</v>
+        <v>أمانة محافظة جدة</v>
       </c>
       <c r="E66" t="str">
-        <v>مؤسسة الصقر للتطوير</v>
+        <v>مجموعة المنارة للتموين</v>
       </c>
       <c r="F66" t="str">
-        <v>1438002</v>
+        <v>1438</v>
       </c>
       <c r="G66" t="str">
         <v>إفادات الأمانات</v>
@@ -1929,22 +1929,22 @@
     </row>
     <row r="67">
       <c r="A67" t="str">
-        <v>177-413620120549</v>
+        <v>177-413040120810</v>
       </c>
       <c r="B67" t="str">
-        <v>2026-09-21</v>
+        <v>2026-08-18</v>
       </c>
       <c r="C67">
-        <v>13818250</v>
+        <v>14303970</v>
       </c>
       <c r="D67" t="str">
-        <v>أمانة محافظة جدة</v>
+        <v>أمانة محافظة الطائف</v>
       </c>
       <c r="E67" t="str">
-        <v>مؤسسة النخبة للاستثمار</v>
+        <v>مجموعة الرمال للتموين</v>
       </c>
       <c r="F67" t="str">
-        <v>1438001</v>
+        <v>1438002</v>
       </c>
       <c r="G67" t="str">
         <v>التعديات واستغلال المواقع (محضر التعدي)</v>
@@ -1955,19 +1955,19 @@
         <v>177-880000182137</v>
       </c>
       <c r="B68" t="str">
-        <v>2025-07-01</v>
+        <v>2025-06-13</v>
       </c>
       <c r="C68">
-        <v>47036730</v>
+        <v>10220080</v>
       </c>
       <c r="D68" t="str">
-        <v>أمانة منطقة الرياض</v>
+        <v>أمانة محافظة جدة</v>
       </c>
       <c r="E68" t="str">
-        <v>مجموعة الخليج العقارية</v>
+        <v>شركة بوابة للمقاولات</v>
       </c>
       <c r="F68" t="str">
-        <v>1438001</v>
+        <v>1438</v>
       </c>
       <c r="G68" t="str">
         <v>إفادات الأمانات</v>
@@ -1975,19 +1975,19 @@
     </row>
     <row r="69">
       <c r="A69" t="str">
-        <v>177-408940122655</v>
+        <v>177-415090119928</v>
       </c>
       <c r="B69" t="str">
-        <v>2026-02-15</v>
+        <v>2025-12-17</v>
       </c>
       <c r="C69">
-        <v>15448310</v>
+        <v>26746230</v>
       </c>
       <c r="D69" t="str">
-        <v>أمانة منطقة مكة المكرمة</v>
+        <v>أمانة المدينة المنورة</v>
       </c>
       <c r="E69" t="str">
-        <v>مجموعة الخليج للنقل</v>
+        <v>شركة الصقر للإعلان</v>
       </c>
       <c r="F69" t="str">
         <v>11442</v>
@@ -2021,22 +2021,22 @@
     </row>
     <row r="71">
       <c r="A71" t="str">
-        <v>177-411260121611</v>
+        <v>177-410660121881</v>
       </c>
       <c r="B71" t="str">
-        <v>2026-05-28</v>
+        <v>2026-04-27</v>
       </c>
       <c r="C71">
-        <v>43821350</v>
+        <v>6579780</v>
       </c>
       <c r="D71" t="str">
-        <v>أمانة منطقة الحدود الشمالية</v>
+        <v>أمانة المنطقة الشرقية</v>
       </c>
       <c r="E71" t="str">
-        <v>شركة بوابة للخدمات</v>
+        <v>شركة الخليج للنقل</v>
       </c>
       <c r="F71" t="str">
-        <v>14155</v>
+        <v>142163</v>
       </c>
       <c r="G71" t="str">
         <v>التعديات واستغلال المواقع (محضر التعدي)</v>
@@ -2044,22 +2044,22 @@
     </row>
     <row r="72">
       <c r="A72" t="str">
-        <v>177-412180121197</v>
+        <v>177-411380121557</v>
       </c>
       <c r="B72" t="str">
-        <v>2026-06-27</v>
+        <v>2026-05-27</v>
       </c>
       <c r="C72">
-        <v>109664050</v>
+        <v>117936510</v>
       </c>
       <c r="D72" t="str">
         <v>أمانة محافظة جدة</v>
       </c>
       <c r="E72" t="str">
-        <v>شركة الخليج للمقاولات</v>
+        <v>مجموعة بوابة للخدمات</v>
       </c>
       <c r="F72" t="str">
-        <v>1438</v>
+        <v>1438002</v>
       </c>
       <c r="G72" t="str">
         <v>إفادات الأمانات</v>
@@ -2070,19 +2070,19 @@
         <v>177-880000063352</v>
       </c>
       <c r="B73" t="str">
-        <v>2025-03-07</v>
+        <v>2025-02-28</v>
       </c>
       <c r="C73">
-        <v>2858610</v>
+        <v>4164930</v>
       </c>
       <c r="D73" t="str">
-        <v>أمانة محافظة جدة</v>
+        <v>أمانة منطقة جازان</v>
       </c>
       <c r="E73" t="str">
-        <v>مجموعة الشروق للاستثمار</v>
+        <v>شركة الواحة للاستثمار</v>
       </c>
       <c r="F73" t="str">
-        <v>1438001</v>
+        <v>11442</v>
       </c>
       <c r="G73" t="str">
         <v>إفادات الأمانات</v>
@@ -2090,22 +2090,22 @@
     </row>
     <row r="74">
       <c r="A74" t="str">
-        <v>177-410770121872</v>
+        <v>177-410530121980</v>
       </c>
       <c r="B74" t="str">
-        <v>2025-06-13</v>
+        <v>2025-05-21</v>
       </c>
       <c r="C74">
-        <v>10220080</v>
+        <v>2629290</v>
       </c>
       <c r="D74" t="str">
-        <v>أمانة محافظة جدة</v>
+        <v>أمانة المنطقة الشرقية</v>
       </c>
       <c r="E74" t="str">
-        <v>شركة بوابة للمقاولات</v>
+        <v>مؤسسة آفاق للإعلان</v>
       </c>
       <c r="F74" t="str">
-        <v>1438</v>
+        <v>11422</v>
       </c>
       <c r="G74" t="str">
         <v>إفادات الأمانات</v>
@@ -2113,22 +2113,22 @@
     </row>
     <row r="75">
       <c r="A75" t="str">
-        <v>177-413660120531</v>
+        <v>177-413600120558</v>
       </c>
       <c r="B75" t="str">
-        <v>2026-09-03</v>
+        <v>2026-09-15</v>
       </c>
       <c r="C75">
-        <v>46305740</v>
+        <v>57928260</v>
       </c>
       <c r="D75" t="str">
         <v>أمانة محافظة جدة</v>
       </c>
       <c r="E75" t="str">
-        <v>مؤسسة الريادة للتشغيل</v>
+        <v>مؤسسة الفجر للتطوير</v>
       </c>
       <c r="F75" t="str">
-        <v>1438002</v>
+        <v>1438</v>
       </c>
       <c r="G75" t="str">
         <v>التعديات واستغلال المواقع (محضر التعدي)</v>
@@ -2182,22 +2182,22 @@
     </row>
     <row r="78">
       <c r="A78" t="str">
-        <v>177-409280122502</v>
+        <v>177-408820122709</v>
       </c>
       <c r="B78" t="str">
-        <v>2026-03-12</v>
+        <v>2026-02-02</v>
       </c>
       <c r="C78">
-        <v>149461930</v>
+        <v>27687520</v>
       </c>
       <c r="D78" t="str">
         <v>أمانة محافظة جدة</v>
       </c>
       <c r="E78" t="str">
-        <v>مؤسسة المنارة للخدمات</v>
+        <v>شركة الندى للتموين</v>
       </c>
       <c r="F78" t="str">
-        <v>1438002</v>
+        <v>11452105</v>
       </c>
       <c r="G78" t="str">
         <v>إفادات الأمانات</v>
@@ -2214,7 +2214,7 @@
         <v>28817380</v>
       </c>
       <c r="D79" t="str">
-        <v>غير محدد الأمانة (لم تُطابق في مكين)</v>
+        <v>أمانة محافظة جدة</v>
       </c>
       <c r="E79" t="str">
         <v>شركة الجزيرة التجارية</v>
@@ -2251,22 +2251,22 @@
     </row>
     <row r="81">
       <c r="A81" t="str">
-        <v>177-412440121080</v>
+        <v>177-411560121476</v>
       </c>
       <c r="B81" t="str">
-        <v>2026-07-19</v>
+        <v>2026-05-24</v>
       </c>
       <c r="C81">
-        <v>12795650</v>
+        <v>1108040</v>
       </c>
       <c r="D81" t="str">
-        <v>أمانة منطقة مكة المكرمة</v>
+        <v>أمانة محافظة الطائف</v>
       </c>
       <c r="E81" t="str">
-        <v>شركة بنيان للاستثمار</v>
+        <v>مجموعة المدار للتموين</v>
       </c>
       <c r="F81" t="str">
-        <v>1421909</v>
+        <v>1438</v>
       </c>
       <c r="G81" t="str">
         <v>إفادات الأمانات</v>
@@ -2277,16 +2277,16 @@
         <v>177-880000079190</v>
       </c>
       <c r="B82" t="str">
-        <v>2025-03-28</v>
+        <v>2025-03-09</v>
       </c>
       <c r="C82">
-        <v>42545000</v>
+        <v>211460090</v>
       </c>
       <c r="D82" t="str">
-        <v>أمانة منطقة الحدود الشمالية</v>
+        <v>أمانة محافظة جدة</v>
       </c>
       <c r="E82" t="str">
-        <v>شركة بوابة للخدمات</v>
+        <v>مجموعة المنارة للتموين</v>
       </c>
       <c r="F82" t="str">
         <v>14155</v>
@@ -2297,22 +2297,22 @@
     </row>
     <row r="83">
       <c r="A83" t="str">
-        <v>177-411410121584</v>
+        <v>177-410810121854</v>
       </c>
       <c r="B83" t="str">
-        <v>2025-07-01</v>
+        <v>2025-06-03</v>
       </c>
       <c r="C83">
-        <v>47036730</v>
+        <v>45909540</v>
       </c>
       <c r="D83" t="str">
-        <v>أمانة منطقة الرياض</v>
+        <v>أمانة محافظة جدة</v>
       </c>
       <c r="E83" t="str">
-        <v>مجموعة الخليج العقارية</v>
+        <v>شركة الفجر للإعلان</v>
       </c>
       <c r="F83" t="str">
-        <v>1438001</v>
+        <v>1438002</v>
       </c>
       <c r="G83" t="str">
         <v>إفادات الأمانات</v>
@@ -2389,22 +2389,22 @@
     </row>
     <row r="87">
       <c r="A87" t="str">
-        <v>177-409340122475</v>
+        <v>177-409260122511</v>
       </c>
       <c r="B87" t="str">
-        <v>2026-03-18</v>
+        <v>2026-03-13</v>
       </c>
       <c r="C87">
-        <v>77837190</v>
+        <v>20695750</v>
       </c>
       <c r="D87" t="str">
-        <v>أمانة المنطقة الشرقية</v>
+        <v>أمانة محافظة جدة</v>
       </c>
       <c r="E87" t="str">
-        <v>شركة واحة التجارية</v>
+        <v>شركة بنيان للمقاولات</v>
       </c>
       <c r="F87" t="str">
-        <v>1438</v>
+        <v>1438001</v>
       </c>
       <c r="G87" t="str">
         <v>إفادات الأمانات</v>
@@ -2458,19 +2458,19 @@
     </row>
     <row r="90">
       <c r="A90" t="str">
-        <v>177-412740120945</v>
+        <v>177-412080121242</v>
       </c>
       <c r="B90" t="str">
-        <v>2026-07-21</v>
+        <v>2026-06-18</v>
       </c>
       <c r="C90">
-        <v>8835840</v>
+        <v>6579780</v>
       </c>
       <c r="D90" t="str">
-        <v>أمانة محافظة جدة</v>
+        <v>أمانة المنطقة الشرقية</v>
       </c>
       <c r="E90" t="str">
-        <v>مؤسسة الأفق التجارية</v>
+        <v>شركة الخليج للنقل</v>
       </c>
       <c r="F90" t="str">
         <v>142163</v>
@@ -2484,16 +2484,16 @@
         <v>177-880000095028</v>
       </c>
       <c r="B91" t="str">
-        <v>2025-03-28</v>
+        <v>2025-03-09</v>
       </c>
       <c r="C91">
-        <v>6388130</v>
+        <v>66992670</v>
       </c>
       <c r="D91" t="str">
-        <v>أمانة المنطقة الشرقية</v>
+        <v>أمانة منطقة عسير</v>
       </c>
       <c r="E91" t="str">
-        <v>شركة الخليج للنقل</v>
+        <v>مجموعة النخبة للمقاولات</v>
       </c>
       <c r="F91" t="str">
         <v>142163</v>
@@ -2504,22 +2504,22 @@
     </row>
     <row r="92">
       <c r="A92" t="str">
-        <v>177-411830121395</v>
+        <v>177-411490121548</v>
       </c>
       <c r="B92" t="str">
-        <v>2025-07-19</v>
+        <v>2025-07-12</v>
       </c>
       <c r="C92">
-        <v>6588870</v>
+        <v>18038390</v>
       </c>
       <c r="D92" t="str">
         <v>أمانة محافظة جدة</v>
       </c>
       <c r="E92" t="str">
-        <v>مجموعة الواحة للتشغيل</v>
+        <v>شركة بوابة للمقاولات</v>
       </c>
       <c r="F92" t="str">
-        <v>11422</v>
+        <v>1438002</v>
       </c>
       <c r="G92" t="str">
         <v>إفادات الأمانات</v>
@@ -2550,19 +2550,19 @@
     </row>
     <row r="94">
       <c r="A94" t="str">
-        <v>177-411370121602</v>
+        <v>177-410670121917</v>
       </c>
       <c r="B94" t="str">
-        <v>2025-06-27</v>
+        <v>2025-05-09</v>
       </c>
       <c r="C94">
-        <v>6388130</v>
+        <v>66992670</v>
       </c>
       <c r="D94" t="str">
-        <v>أمانة المنطقة الشرقية</v>
+        <v>أمانة منطقة عسير</v>
       </c>
       <c r="E94" t="str">
-        <v>شركة الخليج للنقل</v>
+        <v>مؤسسة الصقر للتطوير</v>
       </c>
       <c r="F94" t="str">
         <v>142163</v>
@@ -2573,19 +2573,19 @@
     </row>
     <row r="95">
       <c r="A95" t="str">
-        <v>177-411370121602</v>
+        <v>177-410670121917</v>
       </c>
       <c r="B95" t="str">
-        <v>2025-06-27</v>
+        <v>2025-05-09</v>
       </c>
       <c r="C95">
-        <v>6388130</v>
+        <v>66992670</v>
       </c>
       <c r="D95" t="str">
         <v>أمانة غير معروفة</v>
       </c>
       <c r="E95" t="str">
-        <v>شركة الخليج للنقل</v>
+        <v>مؤسسة الصقر للتطوير</v>
       </c>
       <c r="F95" t="str">
         <v>142163</v>
@@ -2596,19 +2596,19 @@
     </row>
     <row r="96">
       <c r="A96" t="str">
-        <v>177-409960122196</v>
+        <v>177-409320122484</v>
       </c>
       <c r="B96" t="str">
-        <v>2026-04-22</v>
+        <v>2026-03-24</v>
       </c>
       <c r="C96">
-        <v>6077835</v>
+        <v>36602525</v>
       </c>
       <c r="D96" t="str">
         <v>أمانة محافظة جدة</v>
       </c>
       <c r="E96" t="str">
-        <v>شركة الرؤية للاستثمار</v>
+        <v>مؤسسة السحاب التجارية</v>
       </c>
       <c r="F96" t="str">
         <v>1438001</v>
@@ -2619,7 +2619,7 @@
     </row>
     <row r="97">
       <c r="A97" t="str">
-        <v>302-407620123330</v>
+        <v>028-407620123330</v>
       </c>
       <c r="B97" t="str">
         <v>2024-10-03</v>
@@ -2665,19 +2665,19 @@
     </row>
     <row r="99">
       <c r="A99" t="str">
-        <v>177-412800120918</v>
+        <v>177-412180121197</v>
       </c>
       <c r="B99" t="str">
-        <v>2026-07-09</v>
+        <v>2026-07-06</v>
       </c>
       <c r="C99">
-        <v>69002450</v>
+        <v>109664050</v>
       </c>
       <c r="D99" t="str">
-        <v>أمانة منطقة عسير</v>
+        <v>أمانة محافظة جدة</v>
       </c>
       <c r="E99" t="str">
-        <v>مجموعة النخبة للمقاولات</v>
+        <v>شركة الخليج للمقاولات</v>
       </c>
       <c r="F99" t="str">
         <v>9999999</v>
@@ -2691,19 +2691,19 @@
         <v>177-880000110866</v>
       </c>
       <c r="B100" t="str">
-        <v>2025-04-29</v>
+        <v>2025-04-02</v>
       </c>
       <c r="C100">
-        <v>3787410</v>
+        <v>8364210</v>
       </c>
       <c r="D100" t="str">
-        <v>أمانة محافظة جدة</v>
+        <v>أمانة المنطقة الشرقية</v>
       </c>
       <c r="E100" t="str">
-        <v>مجموعة نماء للتطوير</v>
+        <v>مؤسسة المدار للنقل</v>
       </c>
       <c r="F100" t="str">
-        <v>11452105</v>
+        <v>1438</v>
       </c>
       <c r="G100" t="str">
         <v>إفادات الأمانات</v>
@@ -2711,22 +2711,22 @@
     </row>
     <row r="101">
       <c r="A101" t="str">
-        <v>177-412870120927</v>
+        <v>177-411830121395</v>
       </c>
       <c r="B101" t="str">
-        <v>2025-09-19</v>
+        <v>2025-07-19</v>
       </c>
       <c r="C101">
-        <v>151032890</v>
+        <v>6588870</v>
       </c>
       <c r="D101" t="str">
-        <v>أمانة محافظة الطائف</v>
+        <v>أمانة محافظة جدة</v>
       </c>
       <c r="E101" t="str">
-        <v>مؤسسة بوابة للإعلان</v>
+        <v>مجموعة الواحة للتشغيل</v>
       </c>
       <c r="F101" t="str">
-        <v>1438</v>
+        <v>11422</v>
       </c>
       <c r="G101" t="str">
         <v>إفادات الأمانات</v>
@@ -2757,22 +2757,22 @@
     </row>
     <row r="103">
       <c r="A103" t="str">
-        <v>177-413350120711</v>
+        <v>177-411370121602</v>
       </c>
       <c r="B103" t="str">
-        <v>2025-09-09</v>
+        <v>2025-06-27</v>
       </c>
       <c r="C103">
-        <v>217803890</v>
+        <v>6388130</v>
       </c>
       <c r="D103" t="str">
-        <v>أمانة محافظة جدة</v>
+        <v>أمانة المنطقة الشرقية</v>
       </c>
       <c r="E103" t="str">
-        <v>شركة بوابة للخدمات</v>
+        <v>شركة الخليج للنقل</v>
       </c>
       <c r="F103" t="str">
-        <v>14155</v>
+        <v>142163</v>
       </c>
       <c r="G103" t="str">
         <v>التعديات واستغلال المواقع (محضر التعدي)</v>
@@ -2780,22 +2780,22 @@
     </row>
     <row r="104">
       <c r="A104" t="str">
-        <v>177-413350120711</v>
+        <v>177-411370121602</v>
       </c>
       <c r="B104" t="str">
-        <v>2025-09-09</v>
+        <v>2025-06-27</v>
       </c>
       <c r="C104">
-        <v>217803890</v>
+        <v>6388130</v>
       </c>
       <c r="D104" t="str">
         <v>أمانة غير معروفة</v>
       </c>
       <c r="E104" t="str">
-        <v>شركة بوابة للخدمات</v>
+        <v>شركة الخليج للنقل</v>
       </c>
       <c r="F104" t="str">
-        <v>14155</v>
+        <v>142163</v>
       </c>
       <c r="G104" t="str">
         <v>التعديات واستغلال المواقع (محضر التعدي)</v>
@@ -2803,22 +2803,22 @@
     </row>
     <row r="105">
       <c r="A105" t="str">
-        <v>177-410180122097</v>
+        <v>177-409920122214</v>
       </c>
       <c r="B105" t="str">
-        <v>2026-04-22</v>
+        <v>2026-04-21</v>
       </c>
       <c r="C105">
-        <v>25785775</v>
+        <v>35451485</v>
       </c>
       <c r="D105" t="str">
         <v>أمانة محافظة جدة</v>
       </c>
       <c r="E105" t="str">
-        <v>مجموعة الواحة للإعلان</v>
+        <v>شركة الرؤية للإعلان</v>
       </c>
       <c r="F105" t="str">
-        <v>11114</v>
+        <v>1438</v>
       </c>
       <c r="G105" t="str">
         <v>إفادات الأمانات</v>
@@ -2849,22 +2849,22 @@
     </row>
     <row r="107">
       <c r="A107" t="str">
-        <v>177-408510122889</v>
+        <v>177-408470122907</v>
       </c>
       <c r="B107" t="str">
-        <v>2025-02-01</v>
+        <v>2025-02-23</v>
       </c>
       <c r="C107">
-        <v>9600950</v>
+        <v>33373590</v>
       </c>
       <c r="D107" t="str">
         <v>أمانة محافظة جدة</v>
       </c>
       <c r="E107" t="str">
-        <v>مجموعة الرؤية التجارية</v>
+        <v>مجموعة النخبة للتشغيل</v>
       </c>
       <c r="F107" t="str">
-        <v>11442</v>
+        <v>1421909</v>
       </c>
       <c r="G107" t="str">
         <v>إفادات الأمانات</v>
@@ -2872,19 +2872,19 @@
     </row>
     <row r="108">
       <c r="A108" t="str">
-        <v>177-413020120819</v>
+        <v>177-412440121080</v>
       </c>
       <c r="B108" t="str">
-        <v>2026-08-24</v>
+        <v>2026-07-28</v>
       </c>
       <c r="C108">
-        <v>30558260</v>
+        <v>12795650</v>
       </c>
       <c r="D108" t="str">
-        <v>أمانة منطقة عسير</v>
+        <v>أمانة منطقة مكة المكرمة</v>
       </c>
       <c r="E108" t="str">
-        <v>مؤسسة المنارة للإعلان</v>
+        <v>شركة بنيان للاستثمار</v>
       </c>
       <c r="F108" t="str">
         <v>9999999</v>
@@ -2898,19 +2898,19 @@
         <v>177-880000126704</v>
       </c>
       <c r="B109" t="str">
-        <v>2025-05-29</v>
+        <v>2025-04-09</v>
       </c>
       <c r="C109">
-        <v>17067910</v>
+        <v>217803890</v>
       </c>
       <c r="D109" t="str">
         <v>أمانة محافظة جدة</v>
       </c>
       <c r="E109" t="str">
-        <v>مجموعة المنارة للتموين</v>
+        <v>شركة الأفق للتطوير</v>
       </c>
       <c r="F109" t="str">
-        <v>1438</v>
+        <v>14155</v>
       </c>
       <c r="G109" t="str">
         <v>إفادات الأمانات</v>
@@ -2918,22 +2918,22 @@
     </row>
     <row r="110">
       <c r="A110" t="str">
-        <v>177-413750120531</v>
+        <v>177-412870120927</v>
       </c>
       <c r="B110" t="str">
-        <v>2025-10-12</v>
+        <v>2025-09-19</v>
       </c>
       <c r="C110">
-        <v>8767140</v>
+        <v>151032890</v>
       </c>
       <c r="D110" t="str">
-        <v>أمانة منطقة الرياض</v>
+        <v>أمانة محافظة الطائف</v>
       </c>
       <c r="E110" t="str">
-        <v>مؤسسة بنيان العقارية</v>
+        <v>مؤسسة بوابة للإعلان</v>
       </c>
       <c r="F110" t="str">
-        <v>11422</v>
+        <v>1438</v>
       </c>
       <c r="G110" t="str">
         <v>إفادات الأمانات</v>
@@ -2941,22 +2941,22 @@
     </row>
     <row r="111">
       <c r="A111" t="str">
-        <v>177-408510122889</v>
+        <v>177-408470122907</v>
       </c>
       <c r="B111" t="str">
-        <v>2025-02-01</v>
+        <v>2025-02-23</v>
       </c>
       <c r="C111">
-        <v>9600950</v>
+        <v>33373590</v>
       </c>
       <c r="D111" t="str">
         <v>أمانة المدينة المنورة</v>
       </c>
       <c r="E111" t="str">
-        <v>مجموعة الرؤية التجارية</v>
+        <v>مجموعة النخبة للتشغيل</v>
       </c>
       <c r="F111" t="str">
-        <v>11442</v>
+        <v>1421909</v>
       </c>
       <c r="G111" t="str">
         <v>إفادات الأمانات</v>
@@ -2964,22 +2964,22 @@
     </row>
     <row r="112">
       <c r="A112" t="str">
-        <v>177-414630120135</v>
+        <v>177-413350120711</v>
       </c>
       <c r="B112" t="str">
-        <v>2025-11-09</v>
+        <v>2025-09-09</v>
       </c>
       <c r="C112">
-        <v>66992670</v>
+        <v>217803890</v>
       </c>
       <c r="D112" t="str">
-        <v>أمانة منطقة عسير</v>
+        <v>أمانة محافظة جدة</v>
       </c>
       <c r="E112" t="str">
-        <v>مجموعة النخبة للمقاولات</v>
+        <v>شركة بوابة للخدمات</v>
       </c>
       <c r="F112" t="str">
-        <v>142163</v>
+        <v>14155</v>
       </c>
       <c r="G112" t="str">
         <v>التعديات واستغلال المواقع (محضر التعدي)</v>
@@ -3010,22 +3010,22 @@
     </row>
     <row r="114">
       <c r="A114" t="str">
-        <v>177-410940121755</v>
+        <v>177-410000122178</v>
       </c>
       <c r="B114" t="str">
-        <v>2026-05-26</v>
+        <v>2026-04-06</v>
       </c>
       <c r="C114">
-        <v>75106725</v>
+        <v>57345075</v>
       </c>
       <c r="D114" t="str">
         <v>أمانة محافظة جدة</v>
       </c>
       <c r="E114" t="str">
-        <v>مؤسسة الندى العقارية</v>
+        <v>مؤسسة المدار للتطوير</v>
       </c>
       <c r="F114" t="str">
-        <v>1421909</v>
+        <v>1438</v>
       </c>
       <c r="G114" t="str">
         <v>إفادات الأمانات</v>
@@ -3056,22 +3056,22 @@
     </row>
     <row r="116">
       <c r="A116" t="str">
-        <v>177-408930122700</v>
+        <v>177-408570122862</v>
       </c>
       <c r="B116" t="str">
-        <v>2025-03-07</v>
+        <v>2025-02-28</v>
       </c>
       <c r="C116">
-        <v>2858610</v>
+        <v>4164930</v>
       </c>
       <c r="D116" t="str">
-        <v>أمانة محافظة جدة</v>
+        <v>أمانة منطقة جازان</v>
       </c>
       <c r="E116" t="str">
-        <v>مجموعة الشروق للاستثمار</v>
+        <v>شركة الواحة للاستثمار</v>
       </c>
       <c r="F116" t="str">
-        <v>1438001</v>
+        <v>11442</v>
       </c>
       <c r="G116" t="str">
         <v>إفادات الأمانات</v>
@@ -3079,19 +3079,19 @@
     </row>
     <row r="117">
       <c r="A117" t="str">
-        <v>177-413140120765</v>
+        <v>177-412740120945</v>
       </c>
       <c r="B117" t="str">
-        <v>2026-08-14</v>
+        <v>2026-07-30</v>
       </c>
       <c r="C117">
-        <v>35056450</v>
+        <v>8835840</v>
       </c>
       <c r="D117" t="str">
-        <v>أمانة المنطقة الشرقية</v>
+        <v>أمانة محافظة جدة</v>
       </c>
       <c r="E117" t="str">
-        <v>شركة الصقر للخدمات</v>
+        <v>مؤسسة الأفق التجارية</v>
       </c>
       <c r="F117" t="str">
         <v>9999999</v>
@@ -3105,19 +3105,19 @@
         <v>177-880000142542</v>
       </c>
       <c r="B118" t="str">
-        <v>2025-05-21</v>
+        <v>2025-05-29</v>
       </c>
       <c r="C118">
-        <v>2629290</v>
+        <v>17067910</v>
       </c>
       <c r="D118" t="str">
-        <v>أمانة المنطقة الشرقية</v>
+        <v>أمانة محافظة جدة</v>
       </c>
       <c r="E118" t="str">
-        <v>مؤسسة آفاق للإعلان</v>
+        <v>مجموعة المنارة للتموين</v>
       </c>
       <c r="F118" t="str">
-        <v>11422</v>
+        <v>1438</v>
       </c>
       <c r="G118" t="str">
         <v>إفادات الأمانات</v>
@@ -3125,22 +3125,22 @@
     </row>
     <row r="119">
       <c r="A119" t="str">
-        <v>177-414130120360</v>
+        <v>177-413750120531</v>
       </c>
       <c r="B119" t="str">
-        <v>2025-11-21</v>
+        <v>2025-10-12</v>
       </c>
       <c r="C119">
-        <v>174654120</v>
+        <v>8767140</v>
       </c>
       <c r="D119" t="str">
-        <v>أمانة محافظة جدة</v>
+        <v>أمانة منطقة الرياض</v>
       </c>
       <c r="E119" t="str">
-        <v>شركة الرمال العقارية</v>
+        <v>مؤسسة بنيان العقارية</v>
       </c>
       <c r="F119" t="str">
-        <v>1438001</v>
+        <v>11422</v>
       </c>
       <c r="G119" t="str">
         <v>إفادات الأمانات</v>
@@ -3148,22 +3148,22 @@
     </row>
     <row r="120">
       <c r="A120" t="str">
-        <v>177-408930122700</v>
+        <v>177-408570122862</v>
       </c>
       <c r="B120" t="str">
-        <v>2025-03-07</v>
+        <v>2025-02-28</v>
       </c>
       <c r="C120">
-        <v>2858610</v>
+        <v>4164930</v>
       </c>
       <c r="D120" t="str">
-        <v>أمانة المدينة المنورة</v>
+        <v>أمانة منطقة الحدود الشمالية</v>
       </c>
       <c r="E120" t="str">
-        <v>مجموعة الشروق للاستثمار</v>
+        <v>شركة الواحة للاستثمار</v>
       </c>
       <c r="F120" t="str">
-        <v>1438001</v>
+        <v>11442</v>
       </c>
       <c r="G120" t="str">
         <v>إفادات الأمانات</v>
@@ -3171,19 +3171,19 @@
     </row>
     <row r="121">
       <c r="A121" t="str">
-        <v>177-408580122817</v>
+        <v>177-414630120135</v>
       </c>
       <c r="B121" t="str">
-        <v>2026-01-28</v>
+        <v>2025-11-09</v>
       </c>
       <c r="C121">
-        <v>6579780</v>
+        <v>66992670</v>
       </c>
       <c r="D121" t="str">
-        <v>أمانة المنطقة الشرقية</v>
+        <v>أمانة منطقة عسير</v>
       </c>
       <c r="E121" t="str">
-        <v>شركة الخليج للنقل</v>
+        <v>مجموعة النخبة للمقاولات</v>
       </c>
       <c r="F121" t="str">
         <v>142163</v>
@@ -3194,22 +3194,22 @@
     </row>
     <row r="122">
       <c r="A122" t="str">
-        <v>177-411540121485</v>
+        <v>177-410440121980</v>
       </c>
       <c r="B122" t="str">
-        <v>2026-06-13</v>
+        <v>2026-04-25</v>
       </c>
       <c r="C122">
-        <v>222557505</v>
+        <v>18317335</v>
       </c>
       <c r="D122" t="str">
-        <v>أمانة منطقة عسير</v>
+        <v>أمانة محافظة جدة</v>
       </c>
       <c r="E122" t="str">
-        <v>مجموعة آفاق للنقل</v>
+        <v>مؤسسة الدرة للنقل</v>
       </c>
       <c r="F122" t="str">
-        <v>1438002</v>
+        <v>11422</v>
       </c>
       <c r="G122" t="str">
         <v>إفادات الأمانات</v>
@@ -3240,22 +3240,22 @@
     </row>
     <row r="124">
       <c r="A124" t="str">
-        <v>177-409730122340</v>
+        <v>177-409630122385</v>
       </c>
       <c r="B124" t="str">
-        <v>2025-04-29</v>
+        <v>2025-04-02</v>
       </c>
       <c r="C124">
-        <v>3787410</v>
+        <v>8364210</v>
       </c>
       <c r="D124" t="str">
-        <v>أمانة محافظة جدة</v>
+        <v>أمانة المنطقة الشرقية</v>
       </c>
       <c r="E124" t="str">
-        <v>مجموعة نماء للتطوير</v>
+        <v>مؤسسة المدار للنقل</v>
       </c>
       <c r="F124" t="str">
-        <v>11452105</v>
+        <v>1438</v>
       </c>
       <c r="G124" t="str">
         <v>إفادات الأمانات</v>
@@ -3263,10 +3263,10 @@
     </row>
     <row r="125">
       <c r="A125" t="str">
-        <v>177-413520120594</v>
+        <v>177-412800120918</v>
       </c>
       <c r="B125" t="str">
-        <v>2026-08-09</v>
+        <v>2026-07-09</v>
       </c>
       <c r="C125">
         <v>69002450</v>
@@ -3289,19 +3289,19 @@
         <v>177-880000158380</v>
       </c>
       <c r="B126" t="str">
-        <v>2025-06-13</v>
+        <v>2025-05-21</v>
       </c>
       <c r="C126">
-        <v>10220080</v>
+        <v>2629290</v>
       </c>
       <c r="D126" t="str">
-        <v>أمانة محافظة جدة</v>
+        <v>أمانة المنطقة الشرقية</v>
       </c>
       <c r="E126" t="str">
-        <v>شركة بوابة للمقاولات</v>
+        <v>مؤسسة آفاق للإعلان</v>
       </c>
       <c r="F126" t="str">
-        <v>1438</v>
+        <v>11422</v>
       </c>
       <c r="G126" t="str">
         <v>إفادات الأمانات</v>
@@ -3309,22 +3309,22 @@
     </row>
     <row r="127">
       <c r="A127" t="str">
-        <v>177-414830120045</v>
+        <v>177-414130120360</v>
       </c>
       <c r="B127" t="str">
-        <v>2025-12-17</v>
+        <v>2025-11-21</v>
       </c>
       <c r="C127">
-        <v>47137470</v>
+        <v>174654120</v>
       </c>
       <c r="D127" t="str">
-        <v>أمانة منطقة مكة المكرمة</v>
+        <v>أمانة محافظة جدة</v>
       </c>
       <c r="E127" t="str">
-        <v>مجموعة السحاب العقارية</v>
+        <v>شركة الرمال العقارية</v>
       </c>
       <c r="F127" t="str">
-        <v>1438</v>
+        <v>1438001</v>
       </c>
       <c r="G127" t="str">
         <v>إفادات الأمانات</v>
@@ -3355,22 +3355,22 @@
     </row>
     <row r="129">
       <c r="A129" t="str">
-        <v>177-410620121899</v>
+        <v>177-408580122817</v>
       </c>
       <c r="B129" t="str">
-        <v>2026-04-27</v>
+        <v>2026-01-28</v>
       </c>
       <c r="C129">
-        <v>43821350</v>
+        <v>6579780</v>
       </c>
       <c r="D129" t="str">
-        <v>أمانة منطقة الحدود الشمالية</v>
+        <v>أمانة المنطقة الشرقية</v>
       </c>
       <c r="E129" t="str">
-        <v>شركة بوابة للخدمات</v>
+        <v>شركة الخليج للنقل</v>
       </c>
       <c r="F129" t="str">
-        <v>14155</v>
+        <v>142163</v>
       </c>
       <c r="G129" t="str">
         <v>التعديات واستغلال المواقع (محضر التعدي)</v>
@@ -3378,22 +3378,22 @@
     </row>
     <row r="130">
       <c r="A130" t="str">
-        <v>177-412000121278</v>
+        <v>177-410960121746</v>
       </c>
       <c r="B130" t="str">
-        <v>2026-06-29</v>
+        <v>2026-05-30</v>
       </c>
       <c r="C130">
-        <v>8835965</v>
+        <v>7546875</v>
       </c>
       <c r="D130" t="str">
-        <v>أمانة محافظة جدة</v>
+        <v>أمانة المنطقة الشرقية</v>
       </c>
       <c r="E130" t="str">
-        <v>مؤسسة الأفق التجارية</v>
+        <v>مؤسسة الريادة للإعلان</v>
       </c>
       <c r="F130" t="str">
-        <v>142163</v>
+        <v>11100-11105</v>
       </c>
       <c r="G130" t="str">
         <v>إفادات الأمانات</v>
@@ -3424,22 +3424,22 @@
     </row>
     <row r="132">
       <c r="A132" t="str">
-        <v>177-410170122142</v>
+        <v>177-410130122160</v>
       </c>
       <c r="B132" t="str">
-        <v>2025-05-29</v>
+        <v>2025-05-05</v>
       </c>
       <c r="C132">
-        <v>17067910</v>
+        <v>66118220</v>
       </c>
       <c r="D132" t="str">
         <v>أمانة محافظة جدة</v>
       </c>
       <c r="E132" t="str">
-        <v>مجموعة المنارة للتموين</v>
+        <v>شركة الرمال العقارية</v>
       </c>
       <c r="F132" t="str">
-        <v>1438</v>
+        <v>1438002</v>
       </c>
       <c r="G132" t="str">
         <v>إفادات الأمانات</v>
@@ -3447,22 +3447,22 @@
     </row>
     <row r="133">
       <c r="A133" t="str">
-        <v>177-413600120558</v>
+        <v>177-413020120819</v>
       </c>
       <c r="B133" t="str">
-        <v>2026-09-15</v>
+        <v>2026-08-24</v>
       </c>
       <c r="C133">
-        <v>57928260</v>
+        <v>30558260</v>
       </c>
       <c r="D133" t="str">
-        <v>أمانة محافظة جدة</v>
+        <v>أمانة منطقة عسير</v>
       </c>
       <c r="E133" t="str">
-        <v>مؤسسة الفجر للتطوير</v>
+        <v>مؤسسة المنارة للإعلان</v>
       </c>
       <c r="F133" t="str">
-        <v>1438</v>
+        <v>1438002</v>
       </c>
       <c r="G133" t="str">
         <v>التعديات واستغلال المواقع (محضر التعدي)</v>
@@ -3473,16 +3473,16 @@
         <v>177-880000174218</v>
       </c>
       <c r="B134" t="str">
-        <v>2025-06-27</v>
+        <v>2025-05-28</v>
       </c>
       <c r="C134">
         <v>6388130</v>
       </c>
       <c r="D134" t="str">
-        <v>أمانة المنطقة الشرقية</v>
+        <v>أمانة محافظة جدة</v>
       </c>
       <c r="E134" t="str">
-        <v>شركة الخليج للنقل</v>
+        <v>شركة الأفق للتطوير</v>
       </c>
       <c r="F134" t="str">
         <v>142163</v>
@@ -3493,22 +3493,22 @@
     </row>
     <row r="135">
       <c r="A135" t="str">
-        <v>177-407500123303</v>
+        <v>177-414830120045</v>
       </c>
       <c r="B135" t="str">
-        <v>2026-01-08</v>
+        <v>2025-12-17</v>
       </c>
       <c r="C135">
-        <v>83462690</v>
+        <v>47137470</v>
       </c>
       <c r="D135" t="str">
-        <v>أمانة منطقة عسير</v>
+        <v>أمانة منطقة مكة المكرمة</v>
       </c>
       <c r="E135" t="str">
-        <v>مجموعة الخليج للخدمات</v>
+        <v>مجموعة السحاب العقارية</v>
       </c>
       <c r="F135" t="str">
-        <v>1438001</v>
+        <v>1438</v>
       </c>
       <c r="G135" t="str">
         <v>إفادات الأمانات</v>
@@ -3539,22 +3539,22 @@
     </row>
     <row r="137">
       <c r="A137" t="str">
-        <v>177-411220121629</v>
+        <v>177-410620121899</v>
       </c>
       <c r="B137" t="str">
-        <v>2026-05-29</v>
+        <v>2026-04-27</v>
       </c>
       <c r="C137">
-        <v>21569420</v>
+        <v>43821350</v>
       </c>
       <c r="D137" t="str">
-        <v>أمانة محافظة جدة</v>
+        <v>أمانة منطقة الحدود الشمالية</v>
       </c>
       <c r="E137" t="str">
-        <v>شركة الأفق للتطوير</v>
+        <v>شركة بوابة للخدمات</v>
       </c>
       <c r="F137" t="str">
-        <v>142113</v>
+        <v>14155</v>
       </c>
       <c r="G137" t="str">
         <v>التعديات واستغلال المواقع (محضر التعدي)</v>
@@ -3562,22 +3562,22 @@
     </row>
     <row r="138">
       <c r="A138" t="str">
-        <v>177-412160121206</v>
+        <v>177-411320121584</v>
       </c>
       <c r="B138" t="str">
-        <v>2026-07-20</v>
+        <v>2026-05-19</v>
       </c>
       <c r="C138">
-        <v>77693490</v>
+        <v>6579780</v>
       </c>
       <c r="D138" t="str">
-        <v>أمانة محافظة جدة</v>
+        <v>أمانة المنطقة الشرقية</v>
       </c>
       <c r="E138" t="str">
-        <v>شركة الندى للاستثمار</v>
+        <v>شركة الخليج للنقل</v>
       </c>
       <c r="F138" t="str">
-        <v>1438001</v>
+        <v>142163</v>
       </c>
       <c r="G138" t="str">
         <v>إفادات الأمانات</v>
@@ -3588,16 +3588,16 @@
         <v>177-880000055433</v>
       </c>
       <c r="B139" t="str">
-        <v>2025-02-28</v>
+        <v>2025-02-01</v>
       </c>
       <c r="C139">
-        <v>4164930</v>
+        <v>9600950</v>
       </c>
       <c r="D139" t="str">
-        <v>أمانة منطقة جازان</v>
+        <v>أمانة محافظة جدة</v>
       </c>
       <c r="E139" t="str">
-        <v>شركة الواحة للاستثمار</v>
+        <v>مجموعة الرؤية التجارية</v>
       </c>
       <c r="F139" t="str">
         <v>11442</v>
@@ -3608,22 +3608,22 @@
     </row>
     <row r="140">
       <c r="A140" t="str">
-        <v>177-410530121980</v>
+        <v>177-410230122115</v>
       </c>
       <c r="B140" t="str">
-        <v>2025-05-21</v>
+        <v>2025-05-09</v>
       </c>
       <c r="C140">
-        <v>2629290</v>
+        <v>43823000</v>
       </c>
       <c r="D140" t="str">
-        <v>أمانة المنطقة الشرقية</v>
+        <v>أمانة منطقة عسير</v>
       </c>
       <c r="E140" t="str">
-        <v>مؤسسة آفاق للإعلان</v>
+        <v>مؤسسة الصقر للتطوير</v>
       </c>
       <c r="F140" t="str">
-        <v>11422</v>
+        <v>1438002</v>
       </c>
       <c r="G140" t="str">
         <v>إفادات الأمانات</v>
@@ -3631,22 +3631,22 @@
     </row>
     <row r="141">
       <c r="A141" t="str">
-        <v>177-413640120540</v>
+        <v>177-413140120765</v>
       </c>
       <c r="B141" t="str">
-        <v>2026-09-28</v>
+        <v>2026-08-14</v>
       </c>
       <c r="C141">
-        <v>7242840</v>
+        <v>35056450</v>
       </c>
       <c r="D141" t="str">
-        <v>أمانة محافظة جدة</v>
+        <v>أمانة المنطقة الشرقية</v>
       </c>
       <c r="E141" t="str">
-        <v>شركة الصقر للتطوير</v>
+        <v>شركة الصقر للخدمات</v>
       </c>
       <c r="F141" t="str">
-        <v>1438002</v>
+        <v>1421909</v>
       </c>
       <c r="G141" t="str">
         <v>التعديات واستغلال المواقع (محضر التعدي)</v>

</xml_diff>